<commit_message>
feat(okr-unidad): OKR y prioridades por unidad de fisioterapia
- Nueva pestaña 'OKR por unidad' con selector de centro: prioridades
  automáticas por brecha a meta (críticos primero), resultados clave por
  área y matriz comparativa unidades x áreas.
- Híbrido: hoja opcional OKR_Unidades para definir OKR a medida por unidad
  (plantilla .xlsx/.csv incluida; ejemplos reales precargados).
</commit_message>
<xml_diff>
--- a/plantillas/Plantilla_Cuadro_Mando_Fisio_DASE.xlsx
+++ b/plantillas/Plantilla_Cuadro_Mando_Fisio_DASE.xlsx
@@ -9,7 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Unidades" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CMI" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LÉEME" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="OKR_Unidades" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LÉEME" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1992,7 +1993,208 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Periodo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Unidad</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Codigo</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Objetivo</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>KR</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Valor</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Direccion</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Prioridad</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Dic-2025</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Villablanca</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>16014010</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Recuperar la accesibilidad</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Demora de valoración inicial</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>79.15000000000001</v>
+      </c>
+      <c r="G2" t="n">
+        <v>35</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>menor_mejor</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Dic-2025</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Villablanca</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>16014010</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Recuperar la accesibilidad</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>% de población atendida</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2.82</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>mayor_mejor</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>media</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Dic-2025</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ensanche de Vallecas</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>16014210</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mejorar el cumplimiento de cartera</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Cumplimiento de cartera (506/414)</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>48.1</v>
+      </c>
+      <c r="G4" t="n">
+        <v>74.5</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>mayor_mejor</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>alta</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2095,6 +2297,37 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Hoja OKR_Unidades (opcional) — OKR a medida por unidad. Complementa las prioridades automáticas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Periodo, Unidad, Codigo, Objetivo, KR, Valor, Meta, Direccion, Prioridad</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Una fila por Key Result. Agrupa varios KR bajo el mismo 'Objetivo' y 'Unidad' (o 'Codigo').</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Prioridad: alta/media (opcional). Si dejas esta hoja vacía, el cuadro calcula las prioridades solo.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>